<commit_message>
Apply supplied AG colors and logo while preserving workbook layout
</commit_message>
<xml_diff>
--- a/workbooks/Trykkberegning_ror.xlsx
+++ b/workbooks/Trykkberegning_ror.xlsx
@@ -1329,7 +1329,7 @@
     <t xml:space="preserve">TRYKKBEREGNING AV RØR</t>
   </si>
   <si>
-    <t xml:space="preserve">Væsker · én rørstrekning · eksempeldata ved åpning · blå felt er inndata</t>
+    <t xml:space="preserve">Væsker · én rørstrekning · eksempeldata ved åpning · lysegrønne felt er inndata</t>
   </si>
   <si>
     <t xml:space="preserve">1  RØR OG MATERIALE</t>
@@ -2187,7 +2187,7 @@
     <t xml:space="preserve">1. Rør og materiale</t>
   </si>
   <si>
-    <t xml:space="preserve">Velg rørserie, DN/OD, materiale og EN-produktstandard. Oppgi faktisk veggtykkelse. Ved kjent lysåpning kan du overstyre ID. Metrisk OD er ikke en automatisk material- eller veggserie. En svart/grå verdi er beregnet; blå felt er inndata.</t>
+    <t xml:space="preserve">Velg rørserie, DN/OD, materiale og EN-produktstandard. Oppgi faktisk veggtykkelse. Ved kjent lysåpning kan du overstyre ID. Metrisk OD er ikke en automatisk material- eller veggserie. En mørk verdi er beregnet; lysegrønne felt er inndata.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Væske og drift</t>
@@ -2830,7 +2830,7 @@
     <numFmt numFmtId="181" formatCode="0.0000"/>
     <numFmt numFmtId="182" formatCode="0.0"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2863,7 +2863,7 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF617589"/>
+      <color rgb="FF005149"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2878,21 +2878,14 @@
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF20354C"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF086AA5"/>
-      <name val="Calibri"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF617589"/>
+      <color rgb="FF005149"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2907,7 +2900,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF20354C"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2915,7 +2908,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF20354C"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2931,7 +2924,7 @@
     <font>
       <b val="true"/>
       <sz val="11"/>
-      <color rgb="FF086AA5"/>
+      <color rgb="FF005149"/>
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2944,20 +2937,20 @@
     <font>
       <b val="true"/>
       <sz val="18"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
+      <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -2972,7 +2965,7 @@
     <font>
       <u val="single"/>
       <sz val="11"/>
-      <color rgb="FF086AA5"/>
+      <color rgb="FF005149"/>
       <name val="Cambria"/>
       <family val="0"/>
       <charset val="1"/>
@@ -2986,7 +2979,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2995,38 +2988,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF142D4E"/>
-        <bgColor rgb="FF20354C"/>
+        <fgColor rgb="FF022B2A"/>
+        <bgColor rgb="FF1A1C1B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF087F8C"/>
-        <bgColor rgb="FF008080"/>
+        <fgColor rgb="FF005149"/>
+        <bgColor rgb="FF022B2A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE5F2FF"/>
-        <bgColor rgb="FFE1F3EB"/>
+        <fgColor rgb="FFC0FFDE"/>
+        <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF1F5F9"/>
-        <bgColor rgb="FFF9F9F9"/>
+        <fgColor rgb="FFF5FAF6"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE1F3EB"/>
-        <bgColor rgb="FFE5F2FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF0CE"/>
-        <bgColor rgb="FFFFE5E5"/>
+        <fgColor rgb="FFFFF0EB"/>
+        <bgColor rgb="FFF5FAF6"/>
       </patternFill>
     </fill>
   </fills>
@@ -3043,7 +3030,7 @@
       <right/>
       <top/>
       <bottom style="thin">
-        <color rgb="FFD6E1EA"/>
+        <color rgb="FF40C1AC"/>
       </bottom>
       <diagonal/>
     </border>
@@ -3102,19 +3089,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3122,19 +3109,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="169" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3142,7 +3129,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3150,31 +3137,31 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="173" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3182,39 +3169,39 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="178" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="179" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3222,23 +3209,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="180" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="180" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="181" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="181" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3246,23 +3233,23 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="182" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="182" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3279,21 +3266,21 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFE5E5"/>
+          <bgColor rgb="FFFF4B1A"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFFF0CE"/>
+          <bgColor rgb="FFFFF0EB"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFE5F2FF"/>
+          <fgColor rgb="FFC0FFDE"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3301,7 +3288,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF1F5F9"/>
+          <fgColor rgb="FFF5FAF6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3309,7 +3296,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF086AA5"/>
+          <fgColor rgb="FF005149"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3317,7 +3304,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FF20354C"/>
+          <fgColor rgb="FF1A1C1B"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3338,16 +3325,16 @@
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF087F8C"/>
-      <rgbColor rgb="FFF1F5F9"/>
-      <rgbColor rgb="FF878787"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF888888"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF0CE"/>
-      <rgbColor rgb="FFE1F3EB"/>
+      <rgbColor rgb="FFF5FAF6"/>
+      <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF086AA5"/>
+      <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFD9D9D9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
@@ -3358,29 +3345,29 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFE5F2FF"/>
-      <rgbColor rgb="FFD6E1EA"/>
-      <rgbColor rgb="FFF9F9F9"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFC0FFDE"/>
+      <rgbColor rgb="FFFFF0EB"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFE5E5"/>
-      <rgbColor rgb="FF4F81BD"/>
-      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF40C1AC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFCC00"/>
       <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF617589"/>
+      <rgbColor rgb="FFFF4B1A"/>
+      <rgbColor rgb="FF666699"/>
       <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF142D4E"/>
+      <rgbColor rgb="FF005149"/>
       <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF022B2A"/>
       <rgbColor rgb="FF333300"/>
       <rgbColor rgb="FF993300"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF20354C"/>
+      <rgbColor rgb="FF1A1C1B"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -3407,7 +3394,7 @@
             <a:r>
               <a:rPr sz="1800" b="1" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="1A1C1B"/>
                 </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
@@ -3459,9 +3446,12 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="005149"/>
+            </a:solidFill>
             <a:ln w="12600">
               <a:solidFill>
-                <a:srgbClr val="F9F9F9"/>
+                <a:srgbClr val="005149"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3545,11 +3535,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="40265228"/>
-        <c:axId val="18211899"/>
+        <c:axId val="37334958"/>
+        <c:axId val="31883330"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="40265228"/>
+        <c:axId val="37334958"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3562,7 +3552,7 @@
         <c:spPr>
           <a:ln w="9360">
             <a:solidFill>
-              <a:srgbClr val="878787"/>
+              <a:srgbClr val="888888"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3574,7 +3564,7 @@
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="1A1C1B"/>
                 </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
@@ -3582,14 +3572,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="18211899"/>
+        <c:crossAx val="31883330"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="18211899"/>
+        <c:axId val="31883330"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3599,7 +3589,7 @@
           <c:spPr>
             <a:ln w="9360">
               <a:solidFill>
-                <a:srgbClr val="878787"/>
+                <a:srgbClr val="888888"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3620,7 +3610,7 @@
                 <a:r>
                   <a:rPr sz="1000" b="1" u="none" strike="noStrike">
                     <a:solidFill>
-                      <a:srgbClr val="000000"/>
+                      <a:srgbClr val="1A1C1B"/>
                     </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Calibri"/>
@@ -3645,7 +3635,7 @@
         <c:spPr>
           <a:ln w="9360">
             <a:solidFill>
-              <a:srgbClr val="878787"/>
+              <a:srgbClr val="888888"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3657,7 +3647,7 @@
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
                 <a:solidFill>
-                  <a:srgbClr val="000000"/>
+                  <a:srgbClr val="1A1C1B"/>
                 </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
@@ -3665,7 +3655,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40265228"/>
+        <c:crossAx val="37334958"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3942,72 +3932,645 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>390600</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>698760</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Image 2" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10469880" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>5562720</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>7562520</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9087120" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2228760</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4228560</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10193400" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>2228760</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>4228560</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11744280" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>3895560</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5895360</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9675360" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing14.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1943280</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>77400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1476000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>112680</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8568720" y="77400"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>76320</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>948240</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11424240" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>561960</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2561760</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15998040" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>895320</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>2895120</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15062760" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>428760</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>2428560</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14032440" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>2543040</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>1300680</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="26578440" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>3562200</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>5562000</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="24919200" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>162000</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>2161800</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="11439720" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>5610240</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>178920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1618920</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>118800</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="14491440" y="178920"/>
+          <a:ext cx="1999800" cy="225720"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:srgbClr val="1A1C1B"/>
       </a:dk1>
       <a:lt1>
         <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1F497D"/>
+        <a:srgbClr val="022B2A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="EEECE1"/>
+        <a:srgbClr val="F5FAF6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4F81BD"/>
+        <a:srgbClr val="005149"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="C0504D"/>
+        <a:srgbClr val="40C1AC"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9BBB59"/>
+        <a:srgbClr val="FF4B1A"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064A2"/>
+        <a:srgbClr val="C0FFDE"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4BACC6"/>
+        <a:srgbClr val="022B2A"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="F79646"/>
+        <a:srgbClr val="1A1C1B"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000FF"/>
+        <a:srgbClr val="005149"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="800080"/>
+        <a:srgbClr val="005149"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -4147,7 +4710,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:N54"/>
@@ -4965,19 +5528,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19">
-    <dataValidation sqref="E6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>Rorserier</formula1>
     </dataValidation>
-    <dataValidation sqref="E7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>INDIRECT(IF($E$6="Metrisk OD","MetriskeOD","NominelleDN"))</formula1>
     </dataValidation>
-    <dataValidation sqref="E13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>Materialvalg</formula1>
     </dataValidation>
-    <dataValidation sqref="E14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>ENStandarder</formula1>
     </dataValidation>
-    <dataValidation sqref="E20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>Medievalg</formula1>
     </dataValidation>
     <dataValidation sqref="E9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig tall" error="Oppgi et tall mellom 0 og 1000000000.0." type="decimal" operator="between">
@@ -5032,7 +5595,7 @@
       <formula1>-1</formula1>
       <formula2>10000</formula2>
     </dataValidation>
-    <dataValidation sqref="E34" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E34" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>"Hoveddimensjon,Rørstrekk-tabell"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5060,7 +5623,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C54"/>
@@ -5310,13 +5873,14 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E54"/>
@@ -6177,7 +6741,7 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E54"/>
@@ -6420,13 +6984,14 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D54"/>
@@ -6640,13 +7205,14 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF617589"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E40"/>
@@ -7157,6 +7723,7 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7501,7 +8068,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:M54"/>
@@ -8246,7 +8813,7 @@
       <formula1>-273.14</formula1>
       <formula2>10000</formula2>
     </dataValidation>
-    <dataValidation sqref="E17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="E17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>"Nei,Ja"</formula1>
     </dataValidation>
   </dataValidations>
@@ -8257,14 +8824,15 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:L54"/>
@@ -9307,13 +9875,14 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R54"/>
@@ -10961,13 +11530,14 @@
     <oddHeader/>
     <oddFooter>&amp;C&amp;8 R-rdimensjonering | &amp;A | side &amp;P av &amp;N</oddFooter>
   </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:T54"/>
@@ -12774,7 +13344,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6">
-    <dataValidation sqref="A7:A31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="A7:A31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>Bendtyper</formula1>
     </dataValidation>
     <dataValidation sqref="B7:B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig tall" error="Oppgi et tall mellom 0 og 180." type="decimal" operator="between">
@@ -12813,7 +13383,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:AB54"/>
@@ -15387,13 +15957,13 @@
       <formula1>0</formula1>
       <formula2>1000000000.0</formula2>
     </dataValidation>
-    <dataValidation sqref="A7:A31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="A7:A31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>Ventilvalg</formula1>
     </dataValidation>
-    <dataValidation sqref="G7:G31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="G7:G31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>NominelleDN</formula1>
     </dataValidation>
-    <dataValidation sqref="M7:M31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Blå felt kan redigeres." type="list">
+    <dataValidation sqref="M7:M31" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig valg" error="Velg fra listen, eller bruk et felt for egne verdier." promptTitle="Velg verdi" prompt="Bruk nedtrekkslisten. Lysegrønne felt kan redigeres." type="list">
       <formula1>"Nei,Ja"</formula1>
     </dataValidation>
     <dataValidation sqref="H7:H31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Ugyldig tall" error="Oppgi et tall mellom 0 og 1000000000.0." type="decimal" operator="between">
@@ -15428,7 +15998,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J54"/>
@@ -16896,7 +17466,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F54"/>
@@ -17475,7 +18045,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <tabColor rgb="FF087F8C"/>
+    <tabColor rgb="FF005149"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E54"/>

</xml_diff>

<commit_message>
Prevent pressure chart axis label overlap
</commit_message>
<xml_diff>
--- a/workbooks/Trykkberegning_ror.xlsx
+++ b/workbooks/Trykkberegning_ror.xlsx
@@ -2809,7 +2809,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="19">
+  <numFmts count="20">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.000&quot; bar&quot;"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
@@ -2821,16 +2821,17 @@
     <numFmt numFmtId="172" formatCode="0.000&quot; m væskesøyle&quot;"/>
     <numFmt numFmtId="173" formatCode="0.000&quot; bar(g)&quot;"/>
     <numFmt numFmtId="174" formatCode="0.000&quot; bar&quot;;\-0.000&quot; bar&quot;;&quot;&quot;"/>
-    <numFmt numFmtId="175" formatCode="0.00&quot; bar&quot;"/>
-    <numFmt numFmtId="176" formatCode="0.000&quot; MPa&quot;"/>
-    <numFmt numFmtId="177" formatCode="0.0%"/>
-    <numFmt numFmtId="178" formatCode="0.000&quot; mm&quot;"/>
-    <numFmt numFmtId="179" formatCode="0.000000"/>
-    <numFmt numFmtId="180" formatCode="0.000&quot; kPa&quot;"/>
-    <numFmt numFmtId="181" formatCode="0.0000"/>
-    <numFmt numFmtId="182" formatCode="0.0"/>
+    <numFmt numFmtId="175" formatCode="0.###"/>
+    <numFmt numFmtId="176" formatCode="0.00&quot; bar&quot;"/>
+    <numFmt numFmtId="177" formatCode="0.000&quot; MPa&quot;"/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
+    <numFmt numFmtId="179" formatCode="0.000&quot; mm&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.000000"/>
+    <numFmt numFmtId="181" formatCode="0.000&quot; kPa&quot;"/>
+    <numFmt numFmtId="182" formatCode="0.0000"/>
+    <numFmt numFmtId="183" formatCode="0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2943,6 +2944,12 @@
     </font>
     <font>
       <sz val="10"/>
+      <color rgb="FF1A1C1B"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
       <color rgb="FF1A1C1B"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -3177,11 +3184,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="18" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3189,7 +3196,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="178" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3197,11 +3204,11 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="179" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="180" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3217,7 +3224,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="180" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="181" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3225,19 +3232,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="181" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="182" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="180" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="false" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="182" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="183" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3245,7 +3252,7 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3535,11 +3542,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="37334958"/>
-        <c:axId val="31883330"/>
+        <c:axId val="20432413"/>
+        <c:axId val="94732094"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="37334958"/>
+        <c:axId val="20432413"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3572,14 +3579,14 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="31883330"/>
+        <c:crossAx val="94732094"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="31883330"/>
+        <c:axId val="94732094"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3628,7 +3635,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.000&quot; bar&quot;;\-0.000&quot; bar&quot;;&quot;&quot;" sourceLinked="1"/>
+        <c:numFmt formatCode="0.###" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -3641,21 +3648,21 @@
           </a:ln>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr/>
-          <a:lstStyle/>
+          <a:bodyPr rot="-2700000"/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:defRPr sz="900">
                 <a:solidFill>
                   <a:srgbClr val="1A1C1B"/>
                 </a:solidFill>
-                <a:uFillTx/>
-                <a:latin typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
+            <a:r>
+              <a:t/>
+            </a:r>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37334958"/>
+        <c:crossAx val="20432413"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>